<commit_message>
Cuadro de alcance: agregar columnas Observación/riesgo y Documentos de referencia
42 ítems de PCS/SCADA/PSS/ESD/F&G y OT/IT con observación-riesgo y códigos
de documentos de referencia (ACAL-.../normas). Regenerado en Excel, Word y PDF.
</commit_message>
<xml_diff>
--- a/Análisis/Cuadro_Alcance_Control_OT-IT_CPF2.xlsx
+++ b/Análisis/Cuadro_Alcance_Control_OT-IT_CPF2.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen por responsable" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cuadro de Alcance'!$A$4:$G$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cuadro de Alcance'!$A$4:$I$46</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -510,16 +510,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:I50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -569,6 +571,16 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
+          <t>Observación / riesgo</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Documentos de referencia</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
           <t>Páginas</t>
         </is>
       </c>
@@ -591,7 +603,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Tableros del sistema de control de proceso para las nuevas salas remotas INS-007/008. Marcas: Rockwell/Allen Bradley (ControlLogix, Stratix).</t>
+          <t>Tableros del sistema de control de proceso para las nuevas salas remotas INS-007/008. Rockwell/Allen Bradley (ControlLogix, Stratix).</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -605,6 +617,16 @@
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Respetar marca/modelo del Pliego; reserva mín. 20% capacidad / 25% ocupación.</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>ACAL-100-PL-K-105 (Tablero PCS 003); ACAL-100-PL-K-100 (Arq. PCS)</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>P-144, P-408</t>
         </is>
@@ -628,7 +650,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Marshalling para conexionado de campo, reserva mín. 20% capacidad / 25% ocupación; cables FTA.</t>
+          <t>Marshalling para conexionado de campo; cables FTA asociados.</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -642,6 +664,16 @@
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Cantidad según densidad de señales; mantener diseño/arquitectura adoptada.</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>ACAL-100-PL-K-100; Listado de Señales</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>P-144/145, P-408</t>
         </is>
@@ -665,7 +697,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Switches y equipos activos de la red de control en cada sala remota nueva.</t>
+          <t>Switches/equipos activos de la red de control en cada sala remota nueva.</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -679,6 +711,16 @@
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Mantener arquitectura COM existente.</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>ACAL-100-PL-K-109 (Layout COM-003); 226-ACAL-100-PL-K-305 (diag. bloques)</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>P-144</t>
         </is>
@@ -702,7 +744,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Nuevas lógicas (tableros nuevos y señales cableadas a remotas existentes). Subcontrato INAUCO.</t>
+          <t>Nuevas lógicas (tableros nuevos y señales a remotas existentes).</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -716,6 +758,16 @@
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Subcontrato INAUCO obligatorio (lock-in de integrador).</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>GRAL-EI-K-002/003 (ET PCS/SSS); GRAL-ET-K-101</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>P-144/145, P-303</t>
         </is>
@@ -754,7 +806,17 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Ad-67 (01.C.07.03)</t>
+          <t>Suministro reembolsable (Apéndice I); contraste en campo.</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Ad 01.C.07.03; Hojas de Datos INS</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>Ad-67</t>
         </is>
       </c>
     </row>
@@ -776,7 +838,7 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Vienen montados y cableados a cajas de conexión sobre su propio skid (excepto P&amp;ID de proveedores, p.ej. Propak).</t>
+          <t>Vienen montados y cableados a JB sobre su propio skid (excepto P&amp;ID de proveedores, p.ej. Propak).</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -790,6 +852,16 @@
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Riesgo de interfaz skid↔campo; verificar P&amp;ID de proveedores.</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>P&amp;ID de proveedores (Propak); Apéndice A</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>P-408</t>
         </is>
@@ -813,7 +885,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Nuevas pantallas, adecuación de existentes, base OPC, vínculos y documentación. Wonderware/OMI (AVEVA), integrador INAUCO.</t>
+          <t>Nuevas pantallas, adecuación de existentes, base OPC, vínculos y documentación. Wonderware/OMI (AVEVA).</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
@@ -827,6 +899,16 @@
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Mantener Wonderware/OMI + integrador INAUCO; actualizar base OPC.</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>ACAL-000-MO-K-100/101; AARC-100-TI-K-002</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
         <is>
           <t>P-145, P-155</t>
         </is>
@@ -865,6 +947,16 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
+          <t>🚩 Frontera difusa: definir quién garantiza la integración punta a punta.</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Aclaración Anexo 3.1 §3.7 (consulta 42)</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
           <t>P-297</t>
         </is>
       </c>
@@ -887,7 +979,7 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Para el PCS, dentro del subcontrato de AESA. Se anticipa el SIT respecto a IEC-62381.</t>
+          <t>Para el PCS, dentro del subcontrato de AESA.</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
@@ -901,6 +993,16 @@
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Anticipar SIT a taller (IEC-62381 lo ubica post-SAT) para reducir riesgo en sitio.</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>IEC 62381; ACAL-000-MO-K-101</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
         <is>
           <t>P-303</t>
         </is>
@@ -924,7 +1026,7 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Incluida en montaje/programación/integración (sin precio separado en la planilla).</t>
+          <t>Incluida en montaje/programación/integración (sin precio separado).</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
@@ -939,7 +1041,17 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Ad-68 (01.C.07.04.03), P-282</t>
+          <t>🚩 Sin precio separado (incluida) → riesgo de subvaloración / disputa de alcance.</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Ad 01.C.07.04.03</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Ad-68, P-282</t>
         </is>
       </c>
     </row>
@@ -961,7 +1073,7 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Ampliación de HW con tableros ABB, nuevas pantallas y modificación de existentes; desconexión de cargas.</t>
+          <t>Ampliación de HW (tableros ABB), nuevas pantallas y modificación de existentes; desconexión de cargas.</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
@@ -976,7 +1088,17 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>P-144, P-281, Ad-67 (01.C.06.05.18)</t>
+          <t>Mantener ABB; acordar nuevas cargas disponibles para desconexión.</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>021-ACAL-100-PS030-E-302 (Arq.); -E-303 (Topología)</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>P-144, P-281, Ad-67</t>
         </is>
       </c>
     </row>
@@ -1013,6 +1135,16 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
+          <t>Confirmado por consulta de oferente.</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>IEC 61850; 021-ACAL-100-PS030-E-303</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
           <t>P-304</t>
         </is>
       </c>
@@ -1050,6 +1182,16 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
+          <t>🚩 En P-408 rotulado con código del PCS (inconsistencia a reconciliar). FAT si cambia matriz C&amp;E.</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>ACAL-100-PL-K-562/564; ACAL-100-PL-K-551</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
           <t>P-144, P-408</t>
         </is>
       </c>
@@ -1072,7 +1214,7 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Módulos de I/O (según listado de señales + reserva), connector boards, cables FTA y tablero de marshalling completo (sala remota 6).</t>
+          <t>Módulos de I/O (según listado + reserva), connector boards, cables FTA y marshalling completo (sala remota 6).</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
@@ -1086,6 +1228,16 @@
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Única ampliación de HW de seguridad; módulos en rack existente.</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Listado de Señales; ACAL-100-PL-K-100</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>P-145, P-303</t>
         </is>
@@ -1124,6 +1276,16 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
+          <t>Cambios de campo de AESA impactan la configuración → coordinar con PP.</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>Aclaración §3.7 (consulta)</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
           <t>P-303</t>
         </is>
       </c>
@@ -1161,6 +1323,16 @@
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
+          <t>🚩 Misma inconsistencia de código en P-408.</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>ACAL-100-PL-K-552/554; 021-ACAL-100-HD-K-311 (Válvulas ESD)</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
           <t>P-144, P-408</t>
         </is>
       </c>
@@ -1198,6 +1370,16 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
+          <t>A cargo íntegro de AESA.</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>ACAL-100-PL-K-552/554</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
           <t>P-144/145, P-408</t>
         </is>
       </c>
@@ -1220,7 +1402,7 @@
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Excluida del Contratista; PP entrega un controlador demo para las pruebas.</t>
+          <t>Excluida del Contratista; PP entrega un controlador demo para pruebas.</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
@@ -1234,6 +1416,16 @@
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Dependencia de insumos de PP para la integración.</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>Aclaración §3.7</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
         <is>
           <t>P-303</t>
         </is>
@@ -1272,6 +1464,16 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
+          <t>🚩 Verificar plazo de entrega de PP vs. cronograma de pruebas.</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Aclaración (consulta integración)</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
           <t>P-303</t>
         </is>
       </c>
@@ -1309,6 +1511,16 @@
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
+          <t>Define el alcance físico de la detección; condiciona partidas de campo.</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>ISA-TR 84.00.07</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
           <t>P-171, P-242</t>
         </is>
       </c>
@@ -1346,7 +1558,17 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Ad-69 (01.G.08), P-242/250</t>
+          <t>Cantidad/ubicación según estudio F&amp;G.</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>Ad 01.G.08; SED Plano de ubicación de detectores de gas y fuego</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>Ad-69, P-242/250</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1590,7 @@
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Partida 01.G.08 (montaje de alarmas, detectores, pulsadores, sirenas).</t>
+          <t>Partida 01.G.08 (alarmas, detectores, pulsadores, sirenas).</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
@@ -1383,7 +1605,17 @@
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Ad-69 (01.G.08), P-233</t>
+          <t>Apertura de partida solicitada por consulta de oferente.</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>Ad 01.G.08 (solapa B. Detalles)</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>Ad-69, P-233</t>
         </is>
       </c>
     </row>
@@ -1420,6 +1652,16 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
+          <t>🚩 Zona gris de provisión (campo vs. shelter); cerrar en ingeniería.</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>P-232; subcontrato de shelter</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
           <t>P-232</t>
         </is>
       </c>
@@ -1457,7 +1699,17 @@
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Ad-61 (Redef. Rev.1)</t>
+          <t>Cables F&amp;G resistentes al fuego (optimizable con la ingeniería).</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>330-CPF2 — Redefinición de Alcance Rev.1</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>Ad-61</t>
         </is>
       </c>
     </row>
@@ -1479,7 +1731,7 @@
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Se excluye la habilitación de la red de F&amp;G; la auditoría de habilitación está a cargo de PPSA.</t>
+          <t>Se excluye la habilitación de la red de F&amp;G; auditoría de habilitación a cargo de PPSA.</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
@@ -1493,6 +1745,16 @@
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>Riesgo de interfaz en puesta en servicio; coordinar con habilitación AESA.</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>P-234 (Excepciones-Ingeniería)</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
         <is>
           <t>P-234</t>
         </is>
@@ -1531,6 +1793,16 @@
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
+          <t>Base del alcance OT/IT de AESA.</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>001-ACAL-ET-O-100 (ET Disciplina OT)</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
           <t>P-409</t>
         </is>
       </c>
@@ -1568,6 +1840,16 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
+          <t>Plano de cobertura es orientativo; optimizable en ingeniería.</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>001-ACAL-PL-O-200 (cobertura); 001-ACAL-LI-O-203 (equipos)</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
           <t>P-146, P-409</t>
         </is>
       </c>
@@ -1590,7 +1872,7 @@
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Solo desarrollo de ingeniería e instalación de canalizaciones para implementación futura.</t>
+          <t>Solo desarrollo de ingeniería e instalación de canalizaciones para implementación futura por terceros.</t>
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr">
@@ -1604,6 +1886,16 @@
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>No incluye el equipamiento ni la integración (ver fila 29).</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>001-ACAL-ET-O-100 §3.8.1</t>
+        </is>
+      </c>
+      <c r="I32" s="5" t="inlineStr">
         <is>
           <t>P-146</t>
         </is>
@@ -1642,6 +1934,16 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
+          <t>Frontera de responsabilidad con seguridad patrimonial existente.</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>001-ACAL-ET-O-100 §3.8.1</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
           <t>P-146</t>
         </is>
       </c>
@@ -1679,6 +1981,16 @@
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
+          <t>Licencias e integración a IT Local quedan fuera (ver fila 32).</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>001-ACAL-ET-O-100 §3.8.2</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
           <t>P-146/147, P-409</t>
         </is>
       </c>
@@ -1701,7 +2013,7 @@
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Provisión e instalación del rack; tendidos y fusionado certificado de FO/UTP; alimentación redundante; espejos de FO.</t>
+          <t>Provisión e instalación del rack; FO/UTP certificado; alimentación redundante; espejos de FO.</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
@@ -1715,6 +2027,16 @@
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>Concentra todos los servicios IT en salas/shelters.</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>001-ACAL-ET-O-100 §3.8.3</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="inlineStr">
         <is>
           <t>P-147, P-409</t>
         </is>
@@ -1753,6 +2075,16 @@
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
+          <t>🚩 Definir el punto de demarcación IT↔OT y la matriz de interfaz.</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>001-ACAL-ET-O-100 §3.8.2/3.8.3</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
           <t>P-147</t>
         </is>
       </c>
@@ -1775,7 +2107,7 @@
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Provisión, instalación, fusionado y certificación de FO; continuidad del anillo de 24h con caminos disjuntos; arquitectura PRP + redbox / anillos DLR.</t>
+          <t>Provisión, instalación, fusionado y certificación de FO; continuidad del anillo de 24h con caminos disjuntos; PRP + redbox / anillos DLR.</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
@@ -1789,6 +2121,16 @@
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>Mantener filosofía y topología actuales del anillo OT.</t>
+        </is>
+      </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>226-ACAL-102-PL-K-301 (Anillo FO); 001-ACAL-ET-O-100 §3.8.4</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr">
         <is>
           <t>P-147, P-305, P-409</t>
         </is>
@@ -1812,7 +2154,7 @@
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Bandejas portacables, cañeros de PVC, tritubo PEAD para FO.</t>
+          <t>Bandejas portacables, cañeros de PVC Ø160, tritubo PEAD para FO.</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
@@ -1826,6 +2168,16 @@
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>Usar reservas de canalizaciones existentes para acceso a salas.</t>
+        </is>
+      </c>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>226-ACAL-102-PL-K-301</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="inlineStr">
         <is>
           <t>P-409</t>
         </is>
@@ -1849,7 +2201,7 @@
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Según lista de vendors aprobados por PPSA (Cisco, Fortinet, Hirschmann, Stratix, MPLS Hitachi-ABB, Dell, etc.).</t>
+          <t>Según lista de vendors aprobados (Cisco, Fortinet, Hirschmann, Stratix, MPLS Hitachi-ABB, Dell, etc.).</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
@@ -1863,6 +2215,16 @@
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>Solo partners oficiales autorizados por las marcas.</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>Lista de vendors PPSA — §3.8.5</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="inlineStr">
         <is>
           <t>P-148, P-409</t>
         </is>
@@ -1901,6 +2263,16 @@
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
+          <t>🚩 AESA provee los equipos (fila 35) pero NO los configura → ¿quién asegura la red OT?</t>
+        </is>
+      </c>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>Anexo 3.8 (respuestas); P-409</t>
+        </is>
+      </c>
+      <c r="I40" s="5" t="inlineStr">
+        <is>
           <t>P-409</t>
         </is>
       </c>
@@ -1938,6 +2310,16 @@
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
+          <t>🚩 Entregable de ciberseguridad fuera de AESA pese a la cláusula 43.15.</t>
+        </is>
+      </c>
+      <c r="H41" s="5" t="inlineStr">
+        <is>
+          <t>Anexo 3.8; IEC 62443</t>
+        </is>
+      </c>
+      <c r="I41" s="5" t="inlineStr">
+        <is>
           <t>P-409</t>
         </is>
       </c>
@@ -1975,6 +2357,16 @@
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
+          <t>Verificar quién ejecuta estos análisis de red.</t>
+        </is>
+      </c>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>Anexo 3.8</t>
+        </is>
+      </c>
+      <c r="I42" s="5" t="inlineStr">
+        <is>
           <t>P-409</t>
         </is>
       </c>
@@ -2012,6 +2404,16 @@
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
+          <t>🚩 AESA sigue obligada contractualmente pese a la eliminación de los entregables técnicos.</t>
+        </is>
+      </c>
+      <c r="H43" s="5" t="inlineStr">
+        <is>
+          <t>Cláusula 43.15; COBIT / IEC 62443 / RGPD</t>
+        </is>
+      </c>
+      <c r="I43" s="5" t="inlineStr">
+        <is>
           <t>P-118, P-521</t>
         </is>
       </c>
@@ -2049,6 +2451,16 @@
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
+          <t>Catch-all: traslada a AESA todo lo no listado para PP.</t>
+        </is>
+      </c>
+      <c r="H44" s="5" t="inlineStr">
+        <is>
+          <t>Adenda cláusula 3.1.4; Apéndice A</t>
+        </is>
+      </c>
+      <c r="I44" s="5" t="inlineStr">
+        <is>
           <t>Ad-5</t>
         </is>
       </c>
@@ -2086,6 +2498,16 @@
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
+          <t>Riesgo de interfaz: montaje AESA sobre equipo provisto por PP.</t>
+        </is>
+      </c>
+      <c r="H45" s="5" t="inlineStr">
+        <is>
+          <t>Apéndice A</t>
+        </is>
+      </c>
+      <c r="I45" s="5" t="inlineStr">
+        <is>
           <t>P-408, Ad-5</t>
         </is>
       </c>
@@ -2123,6 +2545,16 @@
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
+          <t>Notificar a PP con antelación; FAT de tableros PP si cambia la matriz Causa-Efecto.</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>ACAL-000-MO-K-101; Matriz Causa-Efecto</t>
+        </is>
+      </c>
+      <c r="I46" s="5" t="inlineStr">
+        <is>
           <t>P-145, P-303</t>
         </is>
       </c>
@@ -2157,11 +2589,11 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G46"/>
+  <autoFilter ref="A4:I46"/>
   <mergeCells count="3">
-    <mergeCell ref="A48:G48"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A48:I48"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>